<commit_message>
Rectifies cell values in hdfc mt excel
</commit_message>
<xml_diff>
--- a/app/models/Admin/Hdfc/HdfcMtExcelTemplate.xlsx
+++ b/app/models/Admin/Hdfc/HdfcMtExcelTemplate.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="121">
   <si>
     <t>PAYMENT GATEWAY CHECKLIST</t>
   </si>
@@ -240,6 +240,9 @@
   </si>
   <si>
     <t>CVVV compliant </t>
+  </si>
+  <si>
+    <t>NA</t>
   </si>
   <si>
     <t>CVC2 compliant </t>
@@ -733,7 +736,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="43">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -866,10 +869,6 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -882,10 +881,6 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="165" fontId="12" fillId="2" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -894,32 +889,12 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="16" fillId="0" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="9" fillId="2" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="2" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -1453,39 +1428,45 @@
       <c r="B57" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="C57" s="22"/>
+      <c r="C57" s="22" t="s">
+        <v>64</v>
+      </c>
       <c r="D57" s="17"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="12"/>
       <c r="B58" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="C58" s="22" t="s">
         <v>64</v>
       </c>
-      <c r="C58" s="22"/>
       <c r="D58" s="15"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="12"/>
       <c r="B59" s="13" t="s">
-        <v>65</v>
-      </c>
-      <c r="C59" s="22"/>
+        <v>66</v>
+      </c>
+      <c r="C59" s="22" t="s">
+        <v>64</v>
+      </c>
       <c r="D59" s="17"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="12"/>
       <c r="B60" s="24" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C60" s="22" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D60" s="17"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="12"/>
       <c r="B61" s="16" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C61" s="22"/>
       <c r="D61" s="20"/>
@@ -1493,7 +1474,7 @@
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="12"/>
       <c r="B62" s="28" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C62" s="29"/>
       <c r="D62" s="20"/>
@@ -1501,7 +1482,7 @@
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="12"/>
       <c r="B63" s="13" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C63" s="29"/>
       <c r="D63" s="20"/>
@@ -1509,7 +1490,7 @@
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="12"/>
       <c r="B64" s="13" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C64" s="29"/>
       <c r="D64" s="20"/>
@@ -1517,7 +1498,7 @@
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="12"/>
       <c r="B65" s="13" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C65" s="29"/>
       <c r="D65" s="20"/>
@@ -1525,7 +1506,7 @@
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="12"/>
       <c r="B66" s="13" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C66" s="29"/>
       <c r="D66" s="20"/>
@@ -1533,7 +1514,7 @@
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="12"/>
       <c r="B67" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C67" s="29"/>
       <c r="D67" s="20"/>
@@ -1541,7 +1522,7 @@
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="12"/>
       <c r="B68" s="28" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C68" s="22"/>
       <c r="D68" s="20"/>
@@ -1549,7 +1530,7 @@
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="12"/>
       <c r="B69" s="13" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C69" s="29"/>
       <c r="D69" s="20"/>
@@ -1557,7 +1538,7 @@
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="12"/>
       <c r="B70" s="13" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C70" s="30"/>
       <c r="D70" s="31"/>
@@ -1565,7 +1546,7 @@
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="12"/>
       <c r="B71" s="13" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C71" s="10"/>
       <c r="D71" s="15"/>
@@ -1573,7 +1554,7 @@
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="12"/>
       <c r="B72" s="13" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C72" s="10"/>
       <c r="D72" s="15"/>
@@ -1581,7 +1562,7 @@
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="12"/>
       <c r="B73" s="13" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C73" s="32"/>
       <c r="D73" s="15"/>
@@ -1589,7 +1570,7 @@
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="12"/>
       <c r="B74" s="13" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C74" s="22"/>
       <c r="D74" s="17"/>
@@ -1597,17 +1578,17 @@
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="12"/>
       <c r="B75" s="16" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C75" s="22" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D75" s="17"/>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="12"/>
       <c r="B76" s="16" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C76" s="22" t="s">
         <v>33</v>
@@ -1616,26 +1597,26 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="12"/>
-      <c r="B77" s="33" t="s">
-        <v>84</v>
+      <c r="B77" s="16" t="s">
+        <v>85</v>
       </c>
       <c r="C77" s="22" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D77" s="20"/>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="12"/>
-      <c r="B78" s="33" t="s">
-        <v>85</v>
+      <c r="B78" s="16" t="s">
+        <v>86</v>
       </c>
       <c r="C78" s="22"/>
       <c r="D78" s="20"/>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="12"/>
-      <c r="B79" s="33" t="s">
-        <v>86</v>
+      <c r="B79" s="16" t="s">
+        <v>87</v>
       </c>
       <c r="C79" s="22"/>
       <c r="D79" s="20"/>
@@ -1643,107 +1624,107 @@
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="12"/>
       <c r="B80" s="16" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C80" s="22" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D80" s="20"/>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="12"/>
-      <c r="B81" s="34" t="s">
-        <v>88</v>
+      <c r="B81" s="33" t="s">
+        <v>89</v>
       </c>
       <c r="C81" s="22" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D81" s="17"/>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="12"/>
-      <c r="B82" s="34" t="s">
-        <v>89</v>
+      <c r="B82" s="33" t="s">
+        <v>90</v>
       </c>
       <c r="C82" s="22" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D82" s="17"/>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="12"/>
-      <c r="B83" s="34" t="s">
-        <v>90</v>
+      <c r="B83" s="33" t="s">
+        <v>91</v>
       </c>
       <c r="C83" s="22" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D83" s="17"/>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="12"/>
-      <c r="B84" s="34" t="s">
-        <v>91</v>
+      <c r="B84" s="33" t="s">
+        <v>92</v>
       </c>
       <c r="C84" s="22" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D84" s="17"/>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="12"/>
-      <c r="B85" s="34" t="s">
-        <v>92</v>
+      <c r="B85" s="33" t="s">
+        <v>93</v>
       </c>
       <c r="C85" s="22" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D85" s="17"/>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="12"/>
-      <c r="B86" s="34" t="s">
-        <v>93</v>
+      <c r="B86" s="33" t="s">
+        <v>94</v>
       </c>
       <c r="C86" s="22" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D86" s="17"/>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="12"/>
-      <c r="B87" s="34" t="s">
-        <v>94</v>
+      <c r="B87" s="33" t="s">
+        <v>95</v>
       </c>
       <c r="C87" s="22" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D87" s="17"/>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="12"/>
-      <c r="B88" s="34" t="s">
-        <v>95</v>
+      <c r="B88" s="33" t="s">
+        <v>96</v>
       </c>
       <c r="C88" s="22" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D88" s="17"/>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="12"/>
-      <c r="B89" s="34" t="s">
-        <v>96</v>
+      <c r="B89" s="33" t="s">
+        <v>97</v>
       </c>
       <c r="C89" s="22" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D89" s="17"/>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="12"/>
-      <c r="B90" s="34" t="s">
-        <v>97</v>
+      <c r="B90" s="33" t="s">
+        <v>98</v>
       </c>
       <c r="C90" s="22" t="n">
         <v>10</v>
@@ -1752,278 +1733,278 @@
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="12"/>
-      <c r="B91" s="34" t="s">
-        <v>98</v>
-      </c>
-      <c r="C91" s="35"/>
+      <c r="B91" s="33" t="s">
+        <v>99</v>
+      </c>
+      <c r="C91" s="34"/>
       <c r="D91" s="17"/>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="12"/>
-      <c r="B92" s="36"/>
-      <c r="C92" s="36"/>
+      <c r="B92" s="35"/>
+      <c r="C92" s="35"/>
       <c r="D92" s="17"/>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="12"/>
-      <c r="B93" s="36"/>
-      <c r="C93" s="36"/>
+      <c r="B93" s="35"/>
+      <c r="C93" s="35"/>
       <c r="D93" s="17"/>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="12"/>
-      <c r="B94" s="36"/>
-      <c r="C94" s="36"/>
+      <c r="B94" s="35"/>
+      <c r="C94" s="35"/>
       <c r="D94" s="17"/>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="12"/>
-      <c r="B95" s="36"/>
-      <c r="C95" s="36"/>
+      <c r="B95" s="35"/>
+      <c r="C95" s="35"/>
       <c r="D95" s="17"/>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="12"/>
-      <c r="B96" s="37" t="s">
-        <v>99</v>
-      </c>
-      <c r="C96" s="38"/>
+      <c r="B96" s="24" t="s">
+        <v>100</v>
+      </c>
+      <c r="C96" s="36"/>
       <c r="D96" s="15"/>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="12"/>
-      <c r="B97" s="39" t="s">
-        <v>100</v>
+      <c r="B97" s="37" t="s">
+        <v>101</v>
       </c>
       <c r="C97" s="10"/>
       <c r="D97" s="15"/>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="12"/>
-      <c r="B98" s="40"/>
+      <c r="B98" s="33"/>
       <c r="C98" s="10"/>
       <c r="D98" s="26"/>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="B99" s="41" t="s">
         <v>102</v>
+      </c>
+      <c r="B99" s="9" t="s">
+        <v>103</v>
       </c>
       <c r="C99" s="10"/>
       <c r="D99" s="7"/>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="12"/>
-      <c r="B100" s="42" t="s">
-        <v>103</v>
+      <c r="B100" s="13" t="s">
+        <v>104</v>
       </c>
       <c r="C100" s="14"/>
       <c r="D100" s="15"/>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="12"/>
-      <c r="B101" s="42" t="s">
-        <v>104</v>
+      <c r="B101" s="13" t="s">
+        <v>105</v>
       </c>
       <c r="C101" s="14"/>
       <c r="D101" s="15"/>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="12"/>
-      <c r="B102" s="42" t="s">
-        <v>105</v>
+      <c r="B102" s="13" t="s">
+        <v>106</v>
       </c>
       <c r="C102" s="14"/>
       <c r="D102" s="15"/>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="12"/>
-      <c r="B103" s="42" t="s">
-        <v>106</v>
+      <c r="B103" s="13" t="s">
+        <v>107</v>
       </c>
       <c r="C103" s="10"/>
       <c r="D103" s="15"/>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="12"/>
-      <c r="B104" s="42" t="s">
-        <v>107</v>
+      <c r="B104" s="13" t="s">
+        <v>108</v>
       </c>
       <c r="C104" s="14"/>
       <c r="D104" s="15"/>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="12"/>
-      <c r="B105" s="42" t="s">
-        <v>108</v>
+      <c r="B105" s="13" t="s">
+        <v>109</v>
       </c>
       <c r="C105" s="14"/>
       <c r="D105" s="15"/>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="12"/>
-      <c r="B106" s="42" t="s">
-        <v>109</v>
+      <c r="B106" s="13" t="s">
+        <v>110</v>
       </c>
       <c r="C106" s="14"/>
       <c r="D106" s="15"/>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="12"/>
-      <c r="B107" s="40" t="s">
-        <v>98</v>
+      <c r="B107" s="33" t="s">
+        <v>99</v>
       </c>
       <c r="C107" s="10"/>
       <c r="D107" s="15"/>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="12"/>
-      <c r="B108" s="43"/>
-      <c r="C108" s="43"/>
+      <c r="B108" s="38"/>
+      <c r="C108" s="38"/>
       <c r="D108" s="17"/>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="12"/>
-      <c r="B109" s="43"/>
-      <c r="C109" s="43"/>
+      <c r="B109" s="38"/>
+      <c r="C109" s="38"/>
       <c r="D109" s="17"/>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="12"/>
-      <c r="B110" s="43"/>
-      <c r="C110" s="43"/>
+      <c r="B110" s="38"/>
+      <c r="C110" s="38"/>
       <c r="D110" s="17"/>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="12"/>
-      <c r="B111" s="43"/>
-      <c r="C111" s="43"/>
+      <c r="B111" s="38"/>
+      <c r="C111" s="38"/>
       <c r="D111" s="17"/>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="12"/>
-      <c r="B112" s="43"/>
-      <c r="C112" s="43"/>
+      <c r="B112" s="38"/>
+      <c r="C112" s="38"/>
       <c r="D112" s="17"/>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="12"/>
-      <c r="B113" s="37" t="s">
-        <v>110</v>
-      </c>
-      <c r="C113" s="44"/>
+      <c r="B113" s="24" t="s">
+        <v>111</v>
+      </c>
+      <c r="C113" s="39"/>
       <c r="D113" s="15"/>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="12"/>
-      <c r="B114" s="45"/>
+      <c r="B114" s="18"/>
       <c r="C114" s="10"/>
       <c r="D114" s="15"/>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="B115" s="41" t="s">
         <v>112</v>
+      </c>
+      <c r="B115" s="9" t="s">
+        <v>113</v>
       </c>
       <c r="C115" s="10"/>
       <c r="D115" s="15"/>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="12"/>
-      <c r="B116" s="37" t="s">
-        <v>113</v>
+      <c r="B116" s="24" t="s">
+        <v>114</v>
       </c>
       <c r="C116" s="10"/>
       <c r="D116" s="15"/>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="12"/>
-      <c r="B117" s="42" t="s">
-        <v>114</v>
+      <c r="B117" s="13" t="s">
+        <v>115</v>
       </c>
       <c r="C117" s="10"/>
       <c r="D117" s="15"/>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="12"/>
-      <c r="B118" s="37" t="s">
-        <v>115</v>
+      <c r="B118" s="24" t="s">
+        <v>116</v>
       </c>
       <c r="C118" s="10"/>
       <c r="D118" s="15"/>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="12"/>
-      <c r="B119" s="42" t="s">
-        <v>116</v>
+      <c r="B119" s="13" t="s">
+        <v>117</v>
       </c>
       <c r="C119" s="10"/>
       <c r="D119" s="15"/>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="12"/>
-      <c r="B120" s="42" t="s">
-        <v>117</v>
+      <c r="B120" s="13" t="s">
+        <v>118</v>
       </c>
       <c r="C120" s="10"/>
       <c r="D120" s="15"/>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="12"/>
-      <c r="B121" s="42" t="s">
-        <v>118</v>
+      <c r="B121" s="13" t="s">
+        <v>119</v>
       </c>
       <c r="C121" s="14"/>
       <c r="D121" s="15"/>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="12"/>
-      <c r="B122" s="40" t="s">
-        <v>98</v>
+      <c r="B122" s="33" t="s">
+        <v>99</v>
       </c>
       <c r="C122" s="10"/>
       <c r="D122" s="15"/>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="12"/>
-      <c r="B123" s="46"/>
-      <c r="C123" s="46"/>
+      <c r="B123" s="38"/>
+      <c r="C123" s="38"/>
       <c r="D123" s="17"/>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="12"/>
-      <c r="B124" s="46"/>
-      <c r="C124" s="46"/>
+      <c r="B124" s="38"/>
+      <c r="C124" s="38"/>
       <c r="D124" s="17"/>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="12"/>
-      <c r="B125" s="46"/>
-      <c r="C125" s="46"/>
+      <c r="B125" s="38"/>
+      <c r="C125" s="38"/>
       <c r="D125" s="17"/>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="12"/>
-      <c r="B126" s="46"/>
-      <c r="C126" s="46"/>
+      <c r="B126" s="38"/>
+      <c r="C126" s="38"/>
       <c r="D126" s="17"/>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="12"/>
-      <c r="B127" s="46"/>
-      <c r="C127" s="46"/>
+      <c r="B127" s="38"/>
+      <c r="C127" s="38"/>
       <c r="D127" s="17"/>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="12"/>
       <c r="B128" s="24" t="s">
-        <v>119</v>
-      </c>
-      <c r="C128" s="47"/>
+        <v>120</v>
+      </c>
+      <c r="C128" s="40"/>
       <c r="D128" s="15"/>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2045,8 +2026,8 @@
       <c r="D131" s="15"/>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A132" s="48"/>
-      <c r="B132" s="49"/>
+      <c r="A132" s="41"/>
+      <c r="B132" s="42"/>
       <c r="C132" s="10"/>
       <c r="D132" s="15"/>
     </row>

</xml_diff>